<commit_message>
Poprawa Wag w Scenariuszu 1
</commit_message>
<xml_diff>
--- a/IgniteDigitalization.Server/Initializers/IGNITE_S2_Innowacja.xlsx
+++ b/IgniteDigitalization.Server/Initializers/IGNITE_S2_Innowacja.xlsx
@@ -7,12 +7,14 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feedbacks" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Processes" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CardsWeights" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CardsEnablers" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Boards" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feedbacks" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Processes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CardsWeights" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CardsEnablers" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EconomyRules" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -375,6 +377,168 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>Labels_Up</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>Labels_Right</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>Description_Down</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>Description_Left</t>
+        </is>
+      </c>
+      <c r="F1" s="7" t="inlineStr">
+        <is>
+          <t>Rows</t>
+        </is>
+      </c>
+      <c r="G1" s="7" t="inlineStr">
+        <is>
+          <t>Cols</t>
+        </is>
+      </c>
+      <c r="H1" s="7" t="inlineStr">
+        <is>
+          <t>Border_Color</t>
+        </is>
+      </c>
+      <c r="I1" s="7" t="inlineStr">
+        <is>
+          <t>Cell_Color</t>
+        </is>
+      </c>
+      <c r="J1" s="7" t="inlineStr">
+        <is>
+          <t>Borders_Colors</t>
+        </is>
+      </c>
+      <c r="K1" s="7" t="inlineStr">
+        <is>
+          <t>Cells_Descriptions</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Weryfikacja Rynkowa Innowacji</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Etap komercjalizacji;Trafność przekazu innowacji;Penetracja segmentu;Klarowność kierunku innowacji;</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Rentowność innowacji;Rozpoznawalność innowacji;Lojalność pierwszych klientów;Morale i zaangażowanie;</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>8</v>
+      </c>
+      <c r="G2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>#595959</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>#212121</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>#5faf4c;#f9e44d;#00b8e4;#e32e81</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Zysk;Widoczność;Udział w rynku;Motywacja Zespołu</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Analiza Hipotez</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Podstawowa;Zintegrowana;Inteligentna;Autonomiczna</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Operacyjna;Adaptacyjna;Strategiczna;Innowacyjna</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Automatyzacja Procesów</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Zwinność Procesów</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>8</v>
+      </c>
+      <c r="G3" t="n">
+        <v>8</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>#212121</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>#fefae0</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>#008000;#FFFF00;#FFA500;#FF0000</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
@@ -444,7 +608,7 @@
       </c>
       <c r="K1" s="5" t="inlineStr">
         <is>
-          <t>Card_Phase</t>
+          <t>Card_Phase_Dup</t>
         </is>
       </c>
     </row>
@@ -1322,7 +1486,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1945,7 +2109,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2124,7 +2288,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2307,7 +2471,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2370,10 +2534,10 @@
         <v>1</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="E2" s="3" t="n">
         <v>1</v>
@@ -2400,10 +2564,10 @@
         <v>2</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E3" s="3" t="n">
         <v>1</v>
@@ -2430,10 +2594,10 @@
         <v>3</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E4" s="3" t="n">
         <v>1</v>
@@ -2460,10 +2624,10 @@
         <v>4</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="E5" s="3" t="n">
         <v>1</v>
@@ -2490,10 +2654,10 @@
         <v>1</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E6" s="3" t="n">
         <v>1</v>
@@ -2520,10 +2684,10 @@
         <v>2</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="E7" s="3" t="n">
         <v>1</v>
@@ -2550,10 +2714,10 @@
         <v>3</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="E8" s="3" t="n">
         <v>1</v>
@@ -2580,10 +2744,10 @@
         <v>4</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E9" s="3" t="n">
         <v>1</v>
@@ -2610,10 +2774,10 @@
         <v>1</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E10" s="3" t="n">
         <v>1</v>
@@ -2640,10 +2804,10 @@
         <v>2</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="E11" s="3" t="n">
         <v>1</v>
@@ -2670,10 +2834,10 @@
         <v>3</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="E12" s="3" t="n">
         <v>1</v>
@@ -2700,10 +2864,10 @@
         <v>4</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E13" s="3" t="n">
         <v>1</v>
@@ -2730,10 +2894,10 @@
         <v>1</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E14" s="3" t="n">
         <v>1</v>
@@ -2760,10 +2924,10 @@
         <v>2</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="E15" s="3" t="n">
         <v>1</v>
@@ -2790,10 +2954,10 @@
         <v>3</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="E16" s="3" t="n">
         <v>1</v>
@@ -2820,10 +2984,10 @@
         <v>4</v>
       </c>
       <c r="C17" s="3" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E17" s="3" t="n">
         <v>1</v>
@@ -2850,10 +3014,10 @@
         <v>1</v>
       </c>
       <c r="C18" s="3" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="E18" s="3" t="n">
         <v>1</v>
@@ -2880,10 +3044,10 @@
         <v>2</v>
       </c>
       <c r="C19" s="3" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E19" s="3" t="n">
         <v>1</v>
@@ -2910,10 +3074,10 @@
         <v>3</v>
       </c>
       <c r="C20" s="3" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E20" s="3" t="n">
         <v>1</v>
@@ -2940,10 +3104,10 @@
         <v>4</v>
       </c>
       <c r="C21" s="3" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="E21" s="3" t="n">
         <v>1</v>
@@ -2970,10 +3134,10 @@
         <v>1</v>
       </c>
       <c r="C22" s="3" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="E22" s="3" t="n">
         <v>1</v>
@@ -3000,10 +3164,10 @@
         <v>2</v>
       </c>
       <c r="C23" s="3" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="E23" s="3" t="n">
         <v>1</v>
@@ -3030,10 +3194,10 @@
         <v>3</v>
       </c>
       <c r="C24" s="3" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E24" s="3" t="n">
         <v>1</v>
@@ -3060,10 +3224,10 @@
         <v>4</v>
       </c>
       <c r="C25" s="3" t="n">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="E25" s="3" t="n">
         <v>1</v>
@@ -3090,10 +3254,10 @@
         <v>1</v>
       </c>
       <c r="C26" s="3" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E26" s="3" t="n">
         <v>1</v>
@@ -3120,10 +3284,10 @@
         <v>2</v>
       </c>
       <c r="C27" s="3" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="E27" s="3" t="n">
         <v>1</v>
@@ -3150,10 +3314,10 @@
         <v>3</v>
       </c>
       <c r="C28" s="3" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="E28" s="3" t="n">
         <v>1</v>
@@ -3180,10 +3344,10 @@
         <v>4</v>
       </c>
       <c r="C29" s="3" t="n">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="E29" s="3" t="n">
         <v>1</v>
@@ -3210,10 +3374,10 @@
         <v>1</v>
       </c>
       <c r="C30" s="3" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E30" s="3" t="n">
         <v>1</v>
@@ -3240,10 +3404,10 @@
         <v>2</v>
       </c>
       <c r="C31" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="E31" s="3" t="n">
         <v>1</v>
@@ -3270,10 +3434,10 @@
         <v>3</v>
       </c>
       <c r="C32" s="3" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E32" s="3" t="n">
         <v>1</v>
@@ -3300,10 +3464,10 @@
         <v>4</v>
       </c>
       <c r="C33" s="3" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="E33" s="3" t="n">
         <v>1</v>
@@ -3330,10 +3494,10 @@
         <v>1</v>
       </c>
       <c r="C34" s="3" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E34" s="3" t="n">
         <v>1</v>
@@ -3360,10 +3524,10 @@
         <v>2</v>
       </c>
       <c r="C35" s="3" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="E35" s="3" t="n">
         <v>1</v>
@@ -3390,10 +3554,10 @@
         <v>3</v>
       </c>
       <c r="C36" s="3" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="E36" s="3" t="n">
         <v>1</v>
@@ -3420,10 +3584,10 @@
         <v>4</v>
       </c>
       <c r="C37" s="3" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="E37" s="3" t="n">
         <v>1</v>
@@ -3450,10 +3614,10 @@
         <v>1</v>
       </c>
       <c r="C38" s="3" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="D38" s="3" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="E38" s="3" t="n">
         <v>1</v>
@@ -3480,10 +3644,10 @@
         <v>2</v>
       </c>
       <c r="C39" s="3" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="E39" s="3" t="n">
         <v>1</v>
@@ -3510,10 +3674,10 @@
         <v>3</v>
       </c>
       <c r="C40" s="3" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D40" s="3" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E40" s="3" t="n">
         <v>1</v>
@@ -3540,10 +3704,10 @@
         <v>4</v>
       </c>
       <c r="C41" s="3" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="D41" s="3" t="n">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="E41" s="3" t="n">
         <v>1</v>
@@ -6209,7 +6373,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6247,10 +6411,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="3" t="n">
         <v>11</v>
       </c>
       <c r="C2" s="8" t="inlineStr">
@@ -6258,17 +6422,17 @@
           <t>Crowdfunding wymaga strony docelowej, na którą kierujesz ruch — bez landing page nie masz dokąd odsyłać potencjalnych backerów.</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>PODWÓJNY</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="3" t="n">
         <v>14</v>
       </c>
       <c r="C3" s="8" t="inlineStr">
@@ -6276,17 +6440,17 @@
           <t>Kampania pre-sprzedażowa bez zbudowanej społeczności w social media to krzyczeniew próżnię — nie masz zasięgu ani zaangażowania które napędzą zbiórkę.</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>PODWÓJNY</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="3" t="n">
         <v>17</v>
       </c>
       <c r="C4" s="8" t="inlineStr">
@@ -6294,17 +6458,17 @@
           <t>Nie możesz testować użyteczności czegoś co nie działa — testy użytkowników wymagają działającego prototypu, nie renderingu ani makiety.</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>POJEDYNCZY</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="3" t="n">
         <v>18</v>
       </c>
       <c r="C5" s="8" t="inlineStr">
@@ -6312,17 +6476,17 @@
           <t>Iteracja produktu musi być oparta na danych z testów użytkowników — bez nich zmieniasz produkt na ślepo, nie wiedząc co naprawdę nie działa.</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>POJEDYNCZY</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="3" t="n">
         <v>17</v>
       </c>
       <c r="C6" s="8" t="inlineStr">
@@ -6330,17 +6494,17 @@
           <t>Pilotaż to oddanie prawdziwego urządzenia w ręce klientów — bez działającego prototypu nie masz czego testować w warunkach rzeczywistych.</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>PODWÓJNY</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="3" t="n">
         <v>18</v>
       </c>
       <c r="C7" s="8" t="inlineStr">
@@ -6348,17 +6512,17 @@
           <t>Wysyłanie produktu na pilotaż bez wcześniejszych testów użyteczności to ryzykowanie, że pierwsi klienci dostaną wadliwy sprzęt i staną się krytykami zamiast ambasadorami.</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>PODWÓJNY</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="3" t="n">
         <v>20</v>
       </c>
       <c r="C8" s="8" t="inlineStr">
@@ -6366,17 +6530,17 @@
           <t>Ekspansja na nowy segment bez udanego pilotażu w pierwszym to skalowanie nieznanego — nie wiesz co działało i dlaczego, więc nie masz czego replikować.</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>POJEDYNCZY</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" s="3" t="n">
         <v>26</v>
       </c>
       <c r="C9" s="8" t="inlineStr">
@@ -6384,17 +6548,17 @@
           <t>Model finansowy skalowania bez planu komercjalizacji to kalkulacja w próżni — nie znasz harmonogramu przychodów, kosztów per etap ani momentów zapotrzebowania na kapitał.</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>POJEDYNCZY</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="B10" t="n">
+      <c r="B10" s="3" t="n">
         <v>22</v>
       </c>
       <c r="C10" s="8" t="inlineStr">
@@ -6402,9 +6566,357 @@
           <t>Eco-storytelling bez certyfikacji ekologicznej to greenwashing — w erze Green Claims Directive EU każde twierdzenie o ekologii musi być udokumentowane, a nie tylko ładnie brzmięć.</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>POJEDYNCZY</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="45" customWidth="1" style="4" min="1" max="1"/>
+    <col width="40" customWidth="1" style="4" min="2" max="2"/>
+    <col width="70" customWidth="1" style="4" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>📊  EKONOMIA GRY — IGNITE S2: Innowacja</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Waluta: BITY  |  Zasada ogólna: Zasoby są ograniczone — gracz musi strategicznie wybierać karty i alokować zasoby między hipotezy</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>MAPA 1 — Budżet startowy (Faza Analizy Hipotez)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Budżet startowy</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>24 bity</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Wystarczy na 8–9 z 10 dostępnych kart (koszt karty = 2 bity)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Karty obowiązkowe</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Brak</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Mapa 1 nie ma enablerów — gracz ma pełną swobodę wyboru</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Cel projektowy Mapa 1</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>7–9 kart zagranych</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Gracz nie może zagrać wszystkich — musi priorytetyzować obszary analizy</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>MAPA 2 — Budżet rynkowy (dynamiczny)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Budżet bazowy</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>32 bity</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Każdy zespół startuje na Mapie 2 z tym samym bazowym budżetem</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Bonus przygotowania</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>(kart_PRE / 10) × 12 bitów</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Maksymalny bonus: +12 bitów (jeśli zagrano wszystkie 10 kart PRE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Formuła aplikacji</t>
+        </is>
+      </c>
+      <c r="B12">
+        <f>MIN(44 ; 32 + ROUND((pre/10)*12, 0))</f>
+        <v/>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Aplikacja wylicza budżet Map 2 automatycznie po zakończeniu Map 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Zakres budżetu Mapa 2</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>34–44 bity</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Min: 3 karty PRE → ~36 bitów | Max: 10 kart PRE → 44 bity</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Cel projektowy Mapa 2</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>11–15 kart zagranych</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Gracz musi wybrać strategię: widoczność vs zysk vs rynek vs motywacja</t>
+        </is>
+      </c>
+    </row>
+    <row r="15"/>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>MNOŻNIK PRZYGOTOWANIA — wpływ Mapy 1 na efekty Mapy 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Formuła</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Mnożnik_Wagi = MIN(2,0 ; 1 + kart_PRE_zagranych / 10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>3 kart PRE</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>×1,30</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>minimum — efekty rynkowe o 30% silniejsze niż bazowe</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>5 kart PRE</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>×1,50</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>średnie przygotowanie</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>8 kart PRE</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>×1,80</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>dobre przygotowanie</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>10 kart PRE</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>×2,00</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>maximum — każda karta rynkowa działa 2× silniej</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>MECHANIKA HIPOTEZ INNOWACYJNYCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Pula hipotez startowa</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>10 hipotez do wyboru</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Grill na podczerwieni, grill na wodór, grill solarny, grill pelletowy smart, grill modularny, grill dla kampera, grill profesjonalny HoReCa, grill zero-waste, grill na bioetanol, grill hybrydowy</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Analiza na Mapie 1</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Dowolne spośród 10</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Na Mapie 1 można analizować wszystkie — karty pogłębiają analizę każdej hipotezy</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Wybór do Mapy 2</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2 hipotezy</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Gracze wybierają 2 hipotezy do weryfikacji rynkowej na Mapie 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Rozgrywka per hipoteza</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Mapa 2 działa per hipotezę</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Zasoby Mapy 2 alokowane między 2 hipotezy — koncentracja vs dywersyfikacja to kluczowy wybór</t>
         </is>
       </c>
     </row>

</xml_diff>